<commit_message>
actrualizacion de graphify y errores de [ERR-11] Inconsistencias de alcance y catálogos entre documentos
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/2.1 Product Backlog/Product backlog puntos historia.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/2.1 Product Backlog/Product backlog puntos historia.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Product Backlog con estimación de historias</t>
   </si>
@@ -109,12 +109,51 @@
   </si>
   <si>
     <t>Panel Admin de Usuarios (Web/Desktop)</t>
+  </si>
+  <si>
+    <t>HU-14</t>
+  </si>
+  <si>
+    <t>Finalizar o Cancelar Emergencia</t>
+  </si>
+  <si>
+    <t>HU-15</t>
+  </si>
+  <si>
+    <t>Gestionar Perfil y Credenciales</t>
+  </si>
+  <si>
+    <t>HU-16</t>
+  </si>
+  <si>
+    <t>Adquirir Plan o Cupos (PayPal)</t>
+  </si>
+  <si>
+    <t>HU-17</t>
+  </si>
+  <si>
+    <t>Números Oficiales de Emergencia</t>
+  </si>
+  <si>
+    <t>HU-18</t>
+  </si>
+  <si>
+    <t>Enviar Solicitud de Soporte</t>
+  </si>
+  <si>
+    <t>HU-19</t>
+  </si>
+  <si>
+    <t>Informe Personal de Actividad</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode=""/>
+  </numFmts>
   <fonts count="8">
     <font>
       <sz val="11.0"/>
@@ -160,7 +199,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -171,6 +210,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8F9"/>
+        <bgColor rgb="FFF6F8F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -205,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -215,10 +260,10 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -227,24 +272,33 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -320,7 +374,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:C19" displayName="Tabla_1" name="Tabla_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A6:C25" displayName="Tabla_1" name="Tabla_1" id="1">
   <tableColumns count="3">
     <tableColumn name="Id" id="1"/>
     <tableColumn name="Historia de Usuario" id="2"/>
@@ -588,7 +642,7 @@
         <v>8</v>
       </c>
       <c r="F8" s="7">
-        <f>SUM(C7:C80)</f>
+        <f>SUM(C7:C78)</f>
         <v>44</v>
       </c>
     </row>
@@ -610,7 +664,7 @@
       <c r="B10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="9">
         <v>2.0</v>
       </c>
     </row>
@@ -629,7 +683,7 @@
       <c r="A12" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="5">
@@ -640,7 +694,7 @@
       <c r="A13" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C13" s="5">
@@ -651,7 +705,7 @@
       <c r="A14" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="12" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="5">
@@ -662,7 +716,7 @@
       <c r="A15" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C15" s="5">
@@ -673,7 +727,7 @@
       <c r="A16" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="10" t="s">
         <v>24</v>
       </c>
       <c r="C16" s="5">
@@ -684,7 +738,7 @@
       <c r="A17" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="13" t="s">
         <v>26</v>
       </c>
       <c r="C17" s="8">
@@ -713,79 +767,97 @@
         <v>3.0</v>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="13"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="13"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="13"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
+    <row r="20" ht="35.25" customHeight="1">
+      <c r="A20" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="16"/>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" s="16"/>
+    </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="16"/>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="16"/>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="16"/>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="16"/>
     </row>
     <row r="26">
-      <c r="A26" s="13"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
+      <c r="A26" s="17"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
     </row>
     <row r="27">
-      <c r="A27" s="13"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="13"/>
+      <c r="B27" s="17"/>
     </row>
     <row r="28">
-      <c r="A28" s="13"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
+      <c r="B28" s="17"/>
     </row>
     <row r="29" ht="14.25" customHeight="1">
-      <c r="B29" s="13"/>
+      <c r="B29" s="17"/>
     </row>
     <row r="30" ht="14.25" customHeight="1">
-      <c r="B30" s="13"/>
+      <c r="B30" s="17"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
-      <c r="B31" s="13"/>
+      <c r="B31" s="17"/>
     </row>
     <row r="32" ht="14.25" customHeight="1">
-      <c r="B32" s="13"/>
+      <c r="B32" s="17"/>
     </row>
     <row r="33" ht="14.25" customHeight="1">
-      <c r="B33" s="13"/>
+      <c r="B33" s="17"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
-      <c r="B34" s="13"/>
+      <c r="B34" s="17"/>
     </row>
     <row r="35" ht="14.25" customHeight="1">
-      <c r="B35" s="13"/>
+      <c r="B35" s="17"/>
     </row>
     <row r="36" ht="14.25" customHeight="1">
-      <c r="B36" s="13"/>
-    </row>
-    <row r="37" ht="14.25" customHeight="1">
-      <c r="B37" s="13"/>
-    </row>
-    <row r="38" ht="14.25" customHeight="1">
-      <c r="B38" s="13"/>
-    </row>
+      <c r="B36" s="17"/>
+    </row>
+    <row r="37" ht="14.25" customHeight="1"/>
+    <row r="38" ht="14.25" customHeight="1"/>
     <row r="39" ht="14.25" customHeight="1"/>
     <row r="40" ht="14.25" customHeight="1"/>
     <row r="41" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Actualización de readme y actualización de documentos (NO CORRESPONDIENTES A RAMA "/main")
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/2.1 Product Backlog/Product backlog puntos historia.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/2.1 Product Backlog/Product backlog puntos historia.xlsx
@@ -151,9 +151,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode=""/>
-  </numFmts>
   <fonts count="8">
     <font>
       <sz val="11.0"/>
@@ -250,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -274,9 +271,6 @@
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -289,13 +283,13 @@
     <xf borderId="1" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
@@ -642,8 +636,8 @@
         <v>8</v>
       </c>
       <c r="F8" s="7">
-        <f>SUM(C7:C78)</f>
-        <v>44</v>
+        <f>SUM(C7:C25)</f>
+        <v>62</v>
       </c>
     </row>
     <row r="9" ht="38.25" customHeight="1">
@@ -664,7 +658,7 @@
       <c r="B10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="5">
         <v>2.0</v>
       </c>
     </row>
@@ -683,7 +677,7 @@
       <c r="A12" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="9" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="5">
@@ -694,7 +688,7 @@
       <c r="A13" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="10" t="s">
         <v>18</v>
       </c>
       <c r="C13" s="5">
@@ -705,7 +699,7 @@
       <c r="A14" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="11" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="5">
@@ -716,7 +710,7 @@
       <c r="A15" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="11" t="s">
         <v>22</v>
       </c>
       <c r="C15" s="5">
@@ -727,7 +721,7 @@
       <c r="A16" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="9" t="s">
         <v>24</v>
       </c>
       <c r="C16" s="5">
@@ -738,7 +732,7 @@
       <c r="A17" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="12" t="s">
         <v>26</v>
       </c>
       <c r="C17" s="8">
@@ -768,93 +762,105 @@
       </c>
     </row>
     <row r="20" ht="35.25" customHeight="1">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="16"/>
+      <c r="C20" s="14">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C21" s="16"/>
+      <c r="C21" s="14">
+        <v>4.0</v>
+      </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="15" t="s">
+      <c r="B22" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="16"/>
+      <c r="C22" s="14">
+        <v>5.0</v>
+      </c>
     </row>
     <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C23" s="16"/>
+      <c r="C23" s="14">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="16"/>
+      <c r="C24" s="14">
+        <v>3.0</v>
+      </c>
     </row>
     <row r="25" ht="22.5" customHeight="1">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="16"/>
+      <c r="C25" s="14">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="17"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="17"/>
+      <c r="A26" s="16"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
     </row>
     <row r="27">
-      <c r="B27" s="17"/>
+      <c r="B27" s="16"/>
     </row>
     <row r="28">
-      <c r="B28" s="17"/>
+      <c r="B28" s="16"/>
     </row>
     <row r="29" ht="14.25" customHeight="1">
-      <c r="B29" s="17"/>
+      <c r="B29" s="16"/>
     </row>
     <row r="30" ht="14.25" customHeight="1">
-      <c r="B30" s="17"/>
+      <c r="B30" s="16"/>
     </row>
     <row r="31" ht="14.25" customHeight="1">
-      <c r="B31" s="17"/>
+      <c r="B31" s="16"/>
     </row>
     <row r="32" ht="14.25" customHeight="1">
-      <c r="B32" s="17"/>
+      <c r="B32" s="16"/>
     </row>
     <row r="33" ht="14.25" customHeight="1">
-      <c r="B33" s="17"/>
+      <c r="B33" s="16"/>
     </row>
     <row r="34" ht="14.25" customHeight="1">
-      <c r="B34" s="17"/>
+      <c r="B34" s="16"/>
     </row>
     <row r="35" ht="14.25" customHeight="1">
-      <c r="B35" s="17"/>
+      <c r="B35" s="16"/>
     </row>
     <row r="36" ht="14.25" customHeight="1">
-      <c r="B36" s="17"/>
+      <c r="B36" s="16"/>
     </row>
     <row r="37" ht="14.25" customHeight="1"/>
     <row r="38" ht="14.25" customHeight="1"/>

</xml_diff>